<commit_message>
Pre Market Wed 2026-07-08
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-07-08.xlsx
+++ b/market-prep/Pre Market 2026-07-08.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7500,05</t>
+          <t>7503,85</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29091,00</t>
+          <t>29173,02</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2982,48</t>
+          <t>2982,49</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>52911,99</t>
+          <t>52925,15</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4113,63</t>
+          <t>4105,51</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>60,21</t>
+          <t>59,95</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1639,05</t>
+          <t>1641,70</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>75,69</t>
+          <t>74,16</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>63787,52</t>
+          <t>63380,64</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1788,07</t>
+          <t>1774,68</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>5,01%</t>
+          <t>3,60%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7491,38</t>
+          <t>7503,85</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>